<commit_message>
No 번호 or 문항 in the template; questions shuffled within each type
The 번호 column is gone: the app knows the template's example rows by their
content, so they need no marker (older templates with 번호 = 예시 still
read the same). An example edited in place becomes a question; an unedited
copy further down is reported.

The 문항 tab is gone too: 문법 고르기 and 문법 쓰기 ask the same questions
and count toward scores. Older files with a 문항 sheet still load, and
[엑셀로 받기] writes those questions onto the 문법 tabs.

Questions come a type at a time — words, 문법 고르기, 쓰기, 고치기, 배열 —
and are shuffled within each type; a 고치기 row's find and fix stay
together. [엑셀로 받기] keeps the rows in the order the teacher wrote them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/M2_L7.xlsx
+++ b/public/templates/M2_L7.xlsx
@@ -13,7 +13,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="문법 쓰기" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="문법 고치기" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="문법 배열" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="문항" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,12 +61,6 @@
     <font>
       <name val="맑은 고딕"/>
       <color rgb="00A3A8B4"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="맑은 고딕"/>
-      <b val="1"/>
-      <color rgb="002F6FEB"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -125,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -174,9 +167,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -188,9 +178,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -302,7 +289,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>14</col>
+      <col>13</col>
       <colOff>0</colOff>
       <row>4</row>
       <rowOff>0</rowOff>
@@ -332,7 +319,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>10</col>
+      <col>9</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
@@ -362,7 +349,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>9</col>
+      <col>8</col>
       <colOff>0</colOff>
       <row>2</row>
       <rowOff>0</rowOff>
@@ -392,7 +379,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>9</col>
+      <col>8</col>
       <colOff>0</colOff>
       <row>2</row>
       <rowOff>0</rowOff>
@@ -707,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -796,112 +783,100 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>문항 (선택)</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>위에 없는 문제(반의어 등)를 직접 써요. 점수에는 들어가지 않는 보너스 문제예요.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>알아 두기</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>노란 머리글은 늘 쓰는 칸, 연회색 머리글은 필요할 때 쓰는 칸(보기·정답·해설·지시문·우리말)이에요. 거의 안 쓰는 칸(시간·세트·상태 등)은 오른쪽에 접어 두었어요(표 위 + 를 누르면 보여요).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>노란 머리글은 늘 쓰는 칸, 연회색 머리글은 필요할 때 쓰는 칸(보기·정답·해설·지시문·우리말)이에요. 거의 안 쓰는 칸(시간·세트·상태 등)은 오른쪽에 접어 두었어요(표 위 + 를 누르면 보여요).</t>
+          <t>파란 줄은 예시라서 문제로 나오지 않아요. 예시 줄을 복사해 쓸 때는 내용을 고쳐 쓰면 문제가 돼요.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>파란 '예시' 줄은 문제로 나오지 않아요. 예시 줄을 복사해 쓸 때는 번호 칸의 '예시'를 지우세요.</t>
+          <t>답을 여러 개 인정하려면 | 로 나눠요: [as|so]  ·  Tom is as tall as Jake.|Jake is as tall as Tom.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>답을 여러 개 인정하려면 | 로 나눠요: [as|so]  ·  Tom is as tall as Jake.|Jake is as tall as Tom.</t>
+          <t>문제는 단어 → 문법 고르기 → 쓰기 → 고치기 → 배열 순서로 나오고, 같은 탭 안에서는 앱이 순서를 섞어요.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>문제는 단어 → 문법 탭 순서 → 각 탭의 줄 순서로 나와요.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
           <t>단어장과 문법 탭의 표 오른쪽에 '이렇게 나와요' 화면 예시(프로젝터 · 학생 폰)가 있어요.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>AI로 내 파일 만들기</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>1. AI(챗GPT·Gemini·Claude 등)에 이 파일과 내 자료(본문·단어·문법 문제)를 함께 올려요.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>1. AI(챗GPT·Gemini·Claude 등)에 이 파일과 내 자료(본문·단어·문법 문제)를 함께 올려요.</t>
+          <t>2. 아래 칸의 부탁 글을 복사해 붙여 넣어요.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>2. 아래 칸의 부탁 글을 복사해 붙여 넣어요.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
           <t>3. 받은 파일을 [엑셀 올리기]로 올리고, 미리보기에서 문제와 정답을 확인해요.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="116" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
+    <row r="23" ht="116" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>첨부한 M2_L7.xlsx와 똑같은 형식으로, 첨부한 내 자료의 퀴즈 파일을 만들어 줘.
 - 탭 이름, 머리글, 탭 순서, 열 순서는 그대로 두고, 열을 더하거나 셀을 합치지 마.
-- 각 탭의 파란 '예시' 줄은 그대로 두고, 그 아래 7과 내용만 지우고 내 자료로 채워.
+- 각 탭 맨 위의 파란 예시 줄은 그대로 두고, 그 아래 7과 내용만 지우고 내 자료로 채워.
 - 안내 탭의 표시를 그대로 써: 고르기 (A / B), 쓰기 [답], 고치기 [틀린 말 → 고친 말](표시는 4곳까지), 배열 조각 / 조각(첫 조각도 소문자).
 - 한 줄에 한 문제. 여러 답은 | 로 나누고, 정답은 문장 속 표시와 꼭 맞게 써. 모르는 칸은 비워 둬.
 - 파일 이름은 M2_L8.xlsx처럼 학년_단원으로 해 줘.</t>
         </is>
       </c>
-      <c r="B24" s="7" t="n"/>
+      <c r="B23" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A20:B20"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A24:B24"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A13:B13"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A22:B22"/>
   </mergeCells>
@@ -2245,85 +2220,79 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" style="9" min="1" max="1"/>
-    <col width="38" customWidth="1" style="3" min="2" max="2"/>
-    <col width="9" customWidth="1" style="8" min="3" max="3"/>
+    <col width="38" customWidth="1" style="3" min="1" max="1"/>
+    <col width="9" customWidth="1" style="8" min="2" max="2"/>
+    <col width="11" customWidth="1" style="3" min="3" max="3"/>
     <col width="11" customWidth="1" style="3" min="4" max="4"/>
     <col width="11" customWidth="1" style="3" min="5" max="5"/>
     <col width="11" customWidth="1" style="3" min="6" max="6"/>
-    <col width="11" customWidth="1" style="3" min="7" max="7"/>
-    <col width="13" customWidth="1" style="3" min="8" max="8"/>
+    <col width="13" customWidth="1" style="3" min="7" max="7"/>
+    <col width="12" customWidth="1" style="3" min="8" max="8"/>
     <col width="12" customWidth="1" style="3" min="9" max="9"/>
-    <col width="12" customWidth="1" style="3" min="10" max="10"/>
-    <col hidden="1" outlineLevel="1" width="8" customWidth="1" style="9" min="11" max="13"/>
-    <col width="3" customWidth="1" min="14" max="14"/>
+    <col hidden="1" outlineLevel="1" width="8" customWidth="1" style="9" min="10" max="12"/>
+    <col width="3" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>번호</t>
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>문장</t>
         </is>
       </c>
       <c r="B1" s="10" t="inlineStr">
         <is>
-          <t>문장</t>
-        </is>
-      </c>
-      <c r="C1" s="10" t="inlineStr">
-        <is>
           <t>정답</t>
         </is>
       </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>보기1</t>
+        </is>
+      </c>
       <c r="D1" s="11" t="inlineStr">
         <is>
-          <t>보기1</t>
+          <t>보기2</t>
         </is>
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>보기2</t>
+          <t>보기3</t>
         </is>
       </c>
       <c r="F1" s="11" t="inlineStr">
         <is>
-          <t>보기3</t>
+          <t>보기4</t>
         </is>
       </c>
       <c r="G1" s="11" t="inlineStr">
         <is>
-          <t>보기4</t>
+          <t>해설</t>
         </is>
       </c>
       <c r="H1" s="11" t="inlineStr">
         <is>
-          <t>해설</t>
+          <t>지시문</t>
         </is>
       </c>
       <c r="I1" s="11" t="inlineStr">
         <is>
-          <t>지시문</t>
-        </is>
-      </c>
-      <c r="J1" s="11" t="inlineStr">
-        <is>
           <t>우리말</t>
         </is>
       </c>
+      <c r="J1" s="12" t="inlineStr">
+        <is>
+          <t>시간(초)</t>
+        </is>
+      </c>
       <c r="K1" s="12" t="inlineStr">
         <is>
-          <t>시간(초)</t>
+          <t>세트</t>
         </is>
       </c>
       <c r="L1" s="12" t="inlineStr">
-        <is>
-          <t>세트</t>
-        </is>
-      </c>
-      <c r="M1" s="12" t="inlineStr">
         <is>
           <t>상태</t>
         </is>
@@ -2332,395 +2301,353 @@
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>예시</t>
+          <t>I want (to go / going) home.</t>
         </is>
       </c>
       <c r="B2" s="19" t="inlineStr">
         <is>
-          <t>I want (to go / going) home.</t>
-        </is>
-      </c>
-      <c r="C2" s="20" t="inlineStr">
-        <is>
           <t>to go</t>
         </is>
       </c>
-      <c r="D2" s="19" t="n"/>
-      <c r="E2" s="19" t="n"/>
-      <c r="F2" s="19" t="n"/>
-      <c r="G2" s="19" t="n"/>
-      <c r="H2" s="19" t="inlineStr">
+      <c r="C2" s="18" t="n"/>
+      <c r="D2" s="18" t="n"/>
+      <c r="E2" s="18" t="n"/>
+      <c r="F2" s="18" t="n"/>
+      <c r="G2" s="18" t="inlineStr">
         <is>
           <t>want + to 동사원형</t>
         </is>
       </c>
-      <c r="I2" s="19" t="n"/>
-      <c r="J2" s="19" t="n"/>
-      <c r="K2" s="21" t="n"/>
-      <c r="L2" s="21" t="n"/>
-      <c r="M2" s="21" t="n"/>
+      <c r="H2" s="18" t="n"/>
+      <c r="I2" s="18" t="n"/>
+      <c r="J2" s="20" t="n"/>
+      <c r="K2" s="20" t="n"/>
+      <c r="L2" s="20" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
-        <is>
-          <t>예시</t>
-        </is>
-      </c>
-      <c r="B3" s="19" t="n"/>
-      <c r="C3" s="20" t="inlineStr">
+      <c r="A3" s="18" t="n"/>
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="C3" s="18" t="inlineStr">
         <is>
           <t>He make me laugh.</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
+      <c r="D3" s="18" t="inlineStr">
         <is>
           <t>He makes me laugh.</t>
         </is>
       </c>
-      <c r="F3" s="19" t="n"/>
-      <c r="G3" s="19" t="n"/>
-      <c r="H3" s="19" t="inlineStr">
+      <c r="E3" s="18" t="n"/>
+      <c r="F3" s="18" t="n"/>
+      <c r="G3" s="18" t="inlineStr">
         <is>
           <t>주어가 3인칭 단수면 동사에 -s</t>
         </is>
       </c>
-      <c r="I3" s="19" t="inlineStr">
+      <c r="H3" s="18" t="inlineStr">
         <is>
           <t>바른 문장을 고르세요.</t>
         </is>
       </c>
-      <c r="J3" s="19" t="n"/>
-      <c r="K3" s="21" t="n"/>
-      <c r="L3" s="21" t="n"/>
-      <c r="M3" s="21" t="n"/>
+      <c r="I3" s="18" t="n"/>
+      <c r="J3" s="20" t="n"/>
+      <c r="K3" s="20" t="n"/>
+      <c r="L3" s="20" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="18" t="inlineStr">
         <is>
-          <t>예시</t>
+          <t>Bag A is as heavy as Bag B.</t>
         </is>
       </c>
       <c r="B4" s="19" t="inlineStr">
         <is>
-          <t>Bag A is as heavy as Bag B.</t>
-        </is>
-      </c>
-      <c r="C4" s="20" t="inlineStr">
-        <is>
           <t>O</t>
         </is>
       </c>
-      <c r="D4" s="19" t="n"/>
-      <c r="E4" s="19" t="n"/>
-      <c r="F4" s="19" t="n"/>
-      <c r="G4" s="19" t="n"/>
-      <c r="H4" s="19" t="n"/>
-      <c r="I4" s="19" t="n"/>
-      <c r="J4" s="19" t="inlineStr">
+      <c r="C4" s="18" t="n"/>
+      <c r="D4" s="18" t="n"/>
+      <c r="E4" s="18" t="n"/>
+      <c r="F4" s="18" t="n"/>
+      <c r="G4" s="18" t="n"/>
+      <c r="H4" s="18" t="n"/>
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>가방 A 3kg, 가방 B 3kg</t>
         </is>
       </c>
-      <c r="K4" s="21" t="n"/>
-      <c r="L4" s="21" t="n"/>
-      <c r="M4" s="21" t="n"/>
+      <c r="J4" s="20" t="n"/>
+      <c r="K4" s="20" t="n"/>
+      <c r="L4" s="20" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>The clerk let me (try / to try) on the sneakers.</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>try</t>
         </is>
       </c>
+      <c r="C5" s="14" t="n"/>
       <c r="D5" s="14" t="n"/>
       <c r="E5" s="14" t="n"/>
       <c r="F5" s="14" t="n"/>
-      <c r="G5" s="14" t="n"/>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>let + 목적어 + 동사원형</t>
         </is>
       </c>
+      <c r="H5" s="14" t="n"/>
       <c r="I5" s="14" t="n"/>
-      <c r="J5" s="14" t="n"/>
-      <c r="K5" s="17" t="n"/>
-      <c r="L5" s="16" t="n"/>
-      <c r="M5" s="17" t="n"/>
+      <c r="J5" s="17" t="n"/>
+      <c r="K5" s="16" t="n"/>
+      <c r="L5" s="17" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>My dad made me (water / watering) the plants every morning.</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>water</t>
         </is>
       </c>
+      <c r="C6" s="14" t="n"/>
       <c r="D6" s="14" t="n"/>
       <c r="E6" s="14" t="n"/>
       <c r="F6" s="14" t="n"/>
-      <c r="G6" s="14" t="n"/>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>make + 목적어 + 동사원형</t>
         </is>
       </c>
+      <c r="H6" s="14" t="n"/>
       <c r="I6" s="14" t="n"/>
-      <c r="J6" s="14" t="n"/>
-      <c r="K6" s="17" t="n"/>
-      <c r="L6" s="16" t="n"/>
-      <c r="M6" s="17" t="n"/>
+      <c r="J6" s="17" t="n"/>
+      <c r="K6" s="16" t="n"/>
+      <c r="L6" s="17" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>The teacher had us (exchange / exchanged) our notebooks.</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>exchange</t>
         </is>
       </c>
+      <c r="C7" s="14" t="n"/>
       <c r="D7" s="14" t="n"/>
       <c r="E7" s="14" t="n"/>
       <c r="F7" s="14" t="n"/>
-      <c r="G7" s="14" t="n"/>
-      <c r="H7" s="14" t="inlineStr">
+      <c r="G7" s="14" t="inlineStr">
         <is>
           <t>have + 목적어 + 동사원형</t>
         </is>
       </c>
+      <c r="H7" s="14" t="n"/>
       <c r="I7" s="14" t="n"/>
-      <c r="J7" s="14" t="n"/>
-      <c r="K7" s="17" t="n"/>
-      <c r="L7" s="16" t="n"/>
-      <c r="M7" s="17" t="n"/>
+      <c r="J7" s="17" t="n"/>
+      <c r="K7" s="16" t="n"/>
+      <c r="L7" s="17" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="n">
-        <v>8</v>
-      </c>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="A8" s="14" t="n"/>
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>My mom made me to clean my room.</t>
+        </is>
+      </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>My mom made me to clean my room.</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
           <t>My mom made me clean my room.</t>
         </is>
       </c>
+      <c r="E8" s="14" t="n"/>
       <c r="F8" s="14" t="n"/>
-      <c r="G8" s="14" t="n"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>make + 목적어 + 동사원형 (to 없이)</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr">
         <is>
-          <t>make + 목적어 + 동사원형 (to 없이)</t>
-        </is>
-      </c>
-      <c r="I8" s="14" t="inlineStr">
-        <is>
           <t>어법상 바른 문장을 고르세요.</t>
         </is>
       </c>
-      <c r="J8" s="14" t="n"/>
-      <c r="K8" s="17" t="n"/>
-      <c r="L8" s="16" t="n"/>
-      <c r="M8" s="17" t="n"/>
+      <c r="I8" s="14" t="n"/>
+      <c r="J8" s="17" t="n"/>
+      <c r="K8" s="16" t="n"/>
+      <c r="L8" s="17" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>The flea market lets people (sell / to sell) their secondhand things.</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>sell</t>
         </is>
       </c>
+      <c r="C9" s="14" t="n"/>
       <c r="D9" s="14" t="n"/>
       <c r="E9" s="14" t="n"/>
       <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
-      <c r="H9" s="14" t="inlineStr">
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>let + 목적어 + 동사원형</t>
         </is>
       </c>
+      <c r="H9" s="14" t="n"/>
       <c r="I9" s="14" t="n"/>
-      <c r="J9" s="14" t="n"/>
-      <c r="K9" s="17" t="n"/>
-      <c r="L9" s="16" t="n"/>
-      <c r="M9" s="17" t="n"/>
+      <c r="J9" s="17" t="n"/>
+      <c r="K9" s="16" t="n"/>
+      <c r="L9" s="17" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="n">
-        <v>11</v>
-      </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>This wallet is as (cheap / cheaper) as that one.</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>cheap</t>
         </is>
       </c>
+      <c r="C10" s="14" t="n"/>
       <c r="D10" s="14" t="n"/>
       <c r="E10" s="14" t="n"/>
       <c r="F10" s="14" t="n"/>
-      <c r="G10" s="14" t="n"/>
-      <c r="H10" s="14" t="inlineStr">
+      <c r="G10" s="14" t="inlineStr">
         <is>
           <t>as + 원급 + as</t>
         </is>
       </c>
+      <c r="H10" s="14" t="n"/>
       <c r="I10" s="14" t="n"/>
-      <c r="J10" s="14" t="n"/>
-      <c r="K10" s="17" t="n"/>
-      <c r="L10" s="16" t="n"/>
-      <c r="M10" s="17" t="n"/>
+      <c r="J10" s="17" t="n"/>
+      <c r="K10" s="16" t="n"/>
+      <c r="L10" s="17" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="A11" s="14" t="n"/>
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>My sneakers are as comfortable as yours.</t>
+        </is>
+      </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>My sneakers are as comfortable as yours.</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="inlineStr">
-        <is>
           <t>My sneakers are as more comfortable as yours.</t>
         </is>
       </c>
+      <c r="E11" s="14" t="n"/>
       <c r="F11" s="14" t="n"/>
-      <c r="G11" s="14" t="n"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>as ~ as 사이에는 원급</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>as ~ as 사이에는 원급</t>
-        </is>
-      </c>
-      <c r="I11" s="14" t="inlineStr">
-        <is>
           <t>어법상 바른 문장을 고르세요.</t>
         </is>
       </c>
-      <c r="J11" s="14" t="n"/>
-      <c r="K11" s="17" t="n"/>
-      <c r="L11" s="16" t="n"/>
-      <c r="M11" s="17" t="n"/>
+      <c r="I11" s="14" t="n"/>
+      <c r="J11" s="17" t="n"/>
+      <c r="K11" s="16" t="n"/>
+      <c r="L11" s="17" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="n">
-        <v>16</v>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Mirror A is as expensive as Mirror B.</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
+      <c r="C12" s="14" t="n"/>
       <c r="D12" s="14" t="n"/>
       <c r="E12" s="14" t="n"/>
       <c r="F12" s="14" t="n"/>
-      <c r="G12" s="14" t="n"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>값이 다르니 as expensive as가 아니에요</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr">
         <is>
-          <t>값이 다르니 as expensive as가 아니에요</t>
+          <t>다음 정보를 보고 문장이 맞으면 T, 틀리면 F를 고르세요.</t>
         </is>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
-          <t>다음 정보를 보고 문장이 맞으면 T, 틀리면 F를 고르세요.</t>
-        </is>
-      </c>
-      <c r="J12" s="14" t="inlineStr">
-        <is>
           <t>거울 A: $20 / 거울 B: $30</t>
         </is>
       </c>
-      <c r="K12" s="17" t="n"/>
-      <c r="L12" s="16" t="n"/>
-      <c r="M12" s="17" t="n"/>
+      <c r="J12" s="17" t="n"/>
+      <c r="K12" s="16" t="n"/>
+      <c r="L12" s="17" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="n">
-        <v>18</v>
-      </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>She sings as (beautiful / beautifully) as a singer.</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>beautifully</t>
         </is>
       </c>
+      <c r="C13" s="14" t="n"/>
       <c r="D13" s="14" t="n"/>
       <c r="E13" s="14" t="n"/>
       <c r="F13" s="14" t="n"/>
-      <c r="G13" s="14" t="n"/>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="G13" s="14" t="inlineStr">
         <is>
           <t>sings를 꾸미니 부사 beautifully</t>
         </is>
       </c>
+      <c r="H13" s="14" t="n"/>
       <c r="I13" s="14" t="n"/>
-      <c r="J13" s="14" t="n"/>
-      <c r="K13" s="17" t="n"/>
-      <c r="L13" s="16" t="n"/>
-      <c r="M13" s="17" t="n"/>
+      <c r="J13" s="17" t="n"/>
+      <c r="K13" s="16" t="n"/>
+      <c r="L13" s="17" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="M2:M500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="상태" error="사용, 검토, 보관 중에서 고르세요." type="list">
+    <dataValidation sqref="L2:L500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="상태" error="사용, 검토, 보관 중에서 고르세요." type="list">
       <formula1>"사용,검토,보관"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="시간(초)" error="5~60 사이의 숫자를 쓰거나 비워 두세요." type="whole" operator="between">
+    <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="시간(초)" error="5~60 사이의 숫자를 쓰거나 비워 두세요." type="whole" operator="between">
       <formula1>5</formula1>
       <formula2>60</formula2>
     </dataValidation>
@@ -2736,61 +2663,55 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" style="9" min="1" max="1"/>
-    <col width="40" customWidth="1" style="3" min="2" max="2"/>
-    <col width="18" customWidth="1" style="3" min="3" max="3"/>
-    <col width="16" customWidth="1" style="3" min="4" max="4"/>
+    <col width="40" customWidth="1" style="3" min="1" max="1"/>
+    <col width="18" customWidth="1" style="3" min="2" max="2"/>
+    <col width="16" customWidth="1" style="3" min="3" max="3"/>
+    <col width="14" customWidth="1" style="3" min="4" max="4"/>
     <col width="14" customWidth="1" style="3" min="5" max="5"/>
-    <col width="14" customWidth="1" style="3" min="6" max="6"/>
-    <col hidden="1" outlineLevel="1" width="8" customWidth="1" style="9" min="7" max="9"/>
-    <col width="3" customWidth="1" min="10" max="10"/>
+    <col hidden="1" outlineLevel="1" width="8" customWidth="1" style="9" min="6" max="8"/>
+    <col width="3" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>번호</t>
-        </is>
-      </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>문장</t>
         </is>
       </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>정답</t>
+        </is>
+      </c>
       <c r="C1" s="11" t="inlineStr">
         <is>
-          <t>정답</t>
+          <t>우리말</t>
         </is>
       </c>
       <c r="D1" s="11" t="inlineStr">
         <is>
-          <t>우리말</t>
+          <t>해설</t>
         </is>
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>해설</t>
-        </is>
-      </c>
-      <c r="F1" s="11" t="inlineStr">
-        <is>
           <t>지시문</t>
         </is>
       </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>시간(초)</t>
+        </is>
+      </c>
       <c r="G1" s="12" t="inlineStr">
         <is>
-          <t>시간(초)</t>
+          <t>세트</t>
         </is>
       </c>
       <c r="H1" s="12" t="inlineStr">
-        <is>
-          <t>세트</t>
-        </is>
-      </c>
-      <c r="I1" s="12" t="inlineStr">
         <is>
           <t>상태</t>
         </is>
@@ -2799,225 +2720,197 @@
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>예시</t>
-        </is>
-      </c>
-      <c r="B2" s="19" t="inlineStr">
-        <is>
           <t>He [doesn't] like milk.</t>
         </is>
       </c>
-      <c r="C2" s="19" t="n"/>
-      <c r="D2" s="19" t="inlineStr">
+      <c r="B2" s="18" t="n"/>
+      <c r="C2" s="18" t="inlineStr">
         <is>
           <t>그는 우유를 좋아하지 않는다.</t>
         </is>
       </c>
-      <c r="E2" s="19" t="n"/>
-      <c r="F2" s="19" t="n"/>
-      <c r="G2" s="21" t="n"/>
-      <c r="H2" s="21" t="n"/>
-      <c r="I2" s="21" t="n"/>
+      <c r="D2" s="18" t="n"/>
+      <c r="E2" s="18" t="n"/>
+      <c r="F2" s="20" t="n"/>
+      <c r="G2" s="20" t="n"/>
+      <c r="H2" s="20" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
         <is>
-          <t>예시</t>
-        </is>
-      </c>
-      <c r="B3" s="19" t="inlineStr">
-        <is>
           <t>I like cats. I like dogs.</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>I like cats and dogs.|I like dogs and cats.</t>
         </is>
       </c>
-      <c r="D3" s="19" t="n"/>
-      <c r="E3" s="19" t="n"/>
-      <c r="F3" s="19" t="inlineStr">
+      <c r="C3" s="18" t="n"/>
+      <c r="D3" s="18" t="n"/>
+      <c r="E3" s="18" t="inlineStr">
         <is>
           <t>and로 한 문장을 만드세요.</t>
         </is>
       </c>
-      <c r="G3" s="21" t="n"/>
-      <c r="H3" s="21" t="n"/>
-      <c r="I3" s="21" t="n"/>
+      <c r="F3" s="20" t="n"/>
+      <c r="G3" s="20" t="n"/>
+      <c r="H3" s="20" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>My mom didn’t let me [stay out] late last night. (stay out)</t>
         </is>
       </c>
-      <c r="C4" s="22" t="n"/>
-      <c r="D4" s="14" t="n"/>
+      <c r="B4" s="21" t="n"/>
+      <c r="C4" s="14" t="n"/>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>let + 목적어 + 동사원형</t>
+        </is>
+      </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
+          <t>괄호 안의 말을 알맞은 형태로 바꿔 빈칸에 쓰세요.</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="n"/>
+      <c r="G4" s="16" t="n"/>
+      <c r="H4" s="17" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>The long line made the customers [wait] for an hour. (wait)</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="14" t="n"/>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>make + 목적어 + 동사원형</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>괄호 안의 말을 알맞은 형태로 바꿔 빈칸에 쓰세요.</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="16" t="n"/>
+      <c r="H5" s="17" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>The clerk [let] me [exchange] the wallet.</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>그 점원은 내가 지갑을 교환하게 해 주었다.</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
           <t>let + 목적어 + 동사원형</t>
         </is>
       </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>괄호 안의 말을 알맞은 형태로 바꿔 빈칸에 쓰세요.</t>
-        </is>
-      </c>
-      <c r="G4" s="17" t="n"/>
-      <c r="H4" s="16" t="n"/>
-      <c r="I4" s="17" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="17" t="n">
-        <v>5</v>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>The long line made the customers [wait] for an hour. (wait)</t>
-        </is>
-      </c>
-      <c r="C5" s="22" t="n"/>
-      <c r="D5" s="14" t="n"/>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>make + 목적어 + 동사원형</t>
-        </is>
-      </c>
-      <c r="F5" s="14" t="inlineStr">
-        <is>
-          <t>괄호 안의 말을 알맞은 형태로 바꿔 빈칸에 쓰세요.</t>
-        </is>
-      </c>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="17" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="17" t="n">
-        <v>10</v>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>The clerk [let] me [exchange] the wallet.</t>
-        </is>
-      </c>
-      <c r="C6" s="22" t="n"/>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>그 점원은 내가 지갑을 교환하게 해 주었다.</t>
-        </is>
-      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>let + 목적어 + 동사원형</t>
-        </is>
-      </c>
-      <c r="F6" s="14" t="inlineStr">
-        <is>
           <t>우리말과 같도록 빈칸에 알맞은 말을 쓰세요.</t>
         </is>
       </c>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="16" t="n"/>
-      <c r="I6" s="17" t="n"/>
+      <c r="F6" s="17" t="n"/>
+      <c r="G6" s="16" t="n"/>
+      <c r="H6" s="17" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="n">
-        <v>13</v>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>This scarf is [not] [as|so] expensive [as] that cap.</t>
         </is>
       </c>
-      <c r="C7" s="22" t="n"/>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>이 스카프는 저 모자만큼 비싸지 않다.</t>
+        </is>
+      </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>이 스카프는 저 모자만큼 비싸지 않다.</t>
+          <t>not as(so) + 원급 + as: ~만큼 …하지 않다</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>not as(so) + 원급 + as: ~만큼 …하지 않다</t>
-        </is>
-      </c>
-      <c r="F7" s="14" t="inlineStr">
-        <is>
           <t>우리말과 같도록 빈칸에 알맞은 말을 쓰세요.</t>
         </is>
       </c>
-      <c r="G7" s="17" t="n"/>
-      <c r="H7" s="16" t="n"/>
-      <c r="I7" s="17" t="n"/>
+      <c r="F7" s="17" t="n"/>
+      <c r="G7" s="16" t="n"/>
+      <c r="H7" s="17" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="n">
-        <v>14</v>
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Tom is 160 cm tall. Jake is 160 cm tall, too.</t>
+        </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>Tom is 160 cm tall. Jake is 160 cm tall, too.</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
           <t>Tom is as tall as Jake.|Jake is as tall as Tom.</t>
         </is>
       </c>
-      <c r="D8" s="14" t="n"/>
+      <c r="C8" s="14" t="n"/>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>키가 같으면 as tall as</t>
+        </is>
+      </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>키가 같으면 as tall as</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
           <t>두 문장을 as ~ as를 써서 한 문장으로 만드세요.</t>
         </is>
       </c>
-      <c r="G8" s="17" t="n"/>
-      <c r="H8" s="16" t="n"/>
-      <c r="I8" s="17" t="n"/>
+      <c r="F8" s="17" t="n"/>
+      <c r="G8" s="16" t="n"/>
+      <c r="H8" s="17" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="n">
-        <v>19</v>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>My scarf is [as] warm [as] your jacket.</t>
         </is>
       </c>
-      <c r="C9" s="22" t="n"/>
+      <c r="B9" s="21" t="n"/>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>내 목도리는 네 재킷만큼 따뜻하다.</t>
+        </is>
+      </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>내 목도리는 네 재킷만큼 따뜻하다.</t>
+          <t>as + 원급 + as: ~만큼 …한</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>as + 원급 + as: ~만큼 …한</t>
-        </is>
-      </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
           <t>우리말과 같도록 빈칸에 알맞은 말을 쓰세요.</t>
         </is>
       </c>
-      <c r="G9" s="17" t="n"/>
-      <c r="H9" s="16" t="n"/>
-      <c r="I9" s="17" t="n"/>
+      <c r="F9" s="17" t="n"/>
+      <c r="G9" s="16" t="n"/>
+      <c r="H9" s="17" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="상태" error="사용, 검토, 보관 중에서 고르세요." type="list">
+    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="상태" error="사용, 검토, 보관 중에서 고르세요." type="list">
       <formula1>"사용,검토,보관"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="시간(초)" error="5~60 사이의 숫자를 쓰거나 비워 두세요." type="whole" operator="between">
+    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="시간(초)" error="5~60 사이의 숫자를 쓰거나 비워 두세요." type="whole" operator="between">
       <formula1>5</formula1>
       <formula2>60</formula2>
     </dataValidation>
@@ -3033,55 +2926,49 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" style="9" min="1" max="1"/>
-    <col width="46" customWidth="1" style="3" min="2" max="2"/>
+    <col width="46" customWidth="1" style="3" min="1" max="1"/>
+    <col width="16" customWidth="1" style="3" min="2" max="2"/>
     <col width="16" customWidth="1" style="3" min="3" max="3"/>
-    <col width="16" customWidth="1" style="3" min="4" max="4"/>
-    <col width="14" customWidth="1" style="3" min="5" max="5"/>
-    <col hidden="1" outlineLevel="1" width="8" customWidth="1" style="9" min="6" max="8"/>
-    <col width="3" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" style="3" min="4" max="4"/>
+    <col hidden="1" outlineLevel="1" width="8" customWidth="1" style="9" min="5" max="7"/>
+    <col width="3" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>번호</t>
-        </is>
-      </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>문장</t>
         </is>
       </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>해설</t>
+        </is>
+      </c>
       <c r="C1" s="11" t="inlineStr">
         <is>
-          <t>해설</t>
+          <t>우리말</t>
         </is>
       </c>
       <c r="D1" s="11" t="inlineStr">
         <is>
-          <t>우리말</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
           <t>지시문</t>
         </is>
       </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>시간(초)</t>
+        </is>
+      </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>시간(초)</t>
+          <t>세트</t>
         </is>
       </c>
       <c r="G1" s="12" t="inlineStr">
-        <is>
-          <t>세트</t>
-        </is>
-      </c>
-      <c r="H1" s="12" t="inlineStr">
         <is>
           <t>상태</t>
         </is>
@@ -3090,79 +2977,68 @@
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>예시</t>
-        </is>
-      </c>
-      <c r="B2" s="19" t="inlineStr">
-        <is>
           <t>She [go → goes] to school every day.</t>
         </is>
       </c>
-      <c r="C2" s="19" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>주어가 3인칭 단수면 동사에 -s</t>
         </is>
       </c>
-      <c r="D2" s="19" t="n"/>
-      <c r="E2" s="19" t="n"/>
-      <c r="F2" s="21" t="n"/>
-      <c r="G2" s="21" t="n"/>
-      <c r="H2" s="21" t="n"/>
+      <c r="C2" s="18" t="n"/>
+      <c r="D2" s="18" t="n"/>
+      <c r="E2" s="20" t="n"/>
+      <c r="F2" s="20" t="n"/>
+      <c r="G2" s="20" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="n">
-        <v>6</v>
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>She had her son [to carry → carry] the boxes to the flea market.</t>
+        </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>She had her son [to carry → carry] the boxes to the flea market.</t>
-        </is>
-      </c>
-      <c r="C3" s="14" t="inlineStr">
-        <is>
           <t>have + 목적어 + 동사원형 (to 없이)</t>
         </is>
       </c>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="inlineStr">
         <is>
           <t>어법상 틀린 부분을 찾아 바르게 고치세요.</t>
         </is>
       </c>
-      <c r="F3" s="17" t="n"/>
-      <c r="G3" s="16" t="n"/>
-      <c r="H3" s="17" t="n"/>
+      <c r="E3" s="17" t="n"/>
+      <c r="F3" s="16" t="n"/>
+      <c r="G3" s="17" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="n">
-        <v>15</v>
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>He runs as [fastly → fast] as his brother.</t>
+        </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>He runs as [fastly → fast] as his brother.</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
           <t>fast는 부사도 fast (fastly는 없는 말)</t>
         </is>
       </c>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="C4" s="14" t="n"/>
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>어법상 틀린 부분을 찾아 바르게 고치세요.</t>
         </is>
       </c>
-      <c r="F4" s="17" t="n"/>
-      <c r="G4" s="16" t="n"/>
-      <c r="H4" s="17" t="n"/>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="17" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="상태" error="사용, 검토, 보관 중에서 고르세요." type="list">
+    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="상태" error="사용, 검토, 보관 중에서 고르세요." type="list">
       <formula1>"사용,검토,보관"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="시간(초)" error="5~60 사이의 숫자를 쓰거나 비워 두세요." type="whole" operator="between">
+    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="시간(초)" error="5~60 사이의 숫자를 쓰거나 비워 두세요." type="whole" operator="between">
       <formula1>5</formula1>
       <formula2>60</formula2>
     </dataValidation>
@@ -3178,55 +3054,49 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" style="9" min="1" max="1"/>
-    <col width="42" customWidth="1" style="3" min="2" max="2"/>
-    <col width="22" customWidth="1" style="3" min="3" max="3"/>
+    <col width="42" customWidth="1" style="3" min="1" max="1"/>
+    <col width="22" customWidth="1" style="3" min="2" max="2"/>
+    <col width="14" customWidth="1" style="3" min="3" max="3"/>
     <col width="14" customWidth="1" style="3" min="4" max="4"/>
-    <col width="14" customWidth="1" style="3" min="5" max="5"/>
-    <col hidden="1" outlineLevel="1" width="8" customWidth="1" style="9" min="6" max="8"/>
-    <col width="3" customWidth="1" min="9" max="9"/>
+    <col hidden="1" outlineLevel="1" width="8" customWidth="1" style="9" min="5" max="7"/>
+    <col width="3" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>번호</t>
-        </is>
-      </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>정답 (조각을 / 로)</t>
         </is>
       </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>우리말</t>
+        </is>
+      </c>
       <c r="C1" s="11" t="inlineStr">
         <is>
-          <t>우리말</t>
+          <t>해설</t>
         </is>
       </c>
       <c r="D1" s="11" t="inlineStr">
         <is>
-          <t>해설</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
           <t>지시문</t>
         </is>
       </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>시간(초)</t>
+        </is>
+      </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>시간(초)</t>
+          <t>세트</t>
         </is>
       </c>
       <c r="G1" s="12" t="inlineStr">
-        <is>
-          <t>세트</t>
-        </is>
-      </c>
-      <c r="H1" s="12" t="inlineStr">
         <is>
           <t>상태</t>
         </is>
@@ -3235,103 +3105,89 @@
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>예시</t>
-        </is>
-      </c>
-      <c r="B2" s="19" t="inlineStr">
-        <is>
           <t>my mom / makes / me / drink / milk / every day</t>
         </is>
       </c>
-      <c r="C2" s="19" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>엄마는 내가 매일 우유를 마시게 하신다.</t>
         </is>
       </c>
-      <c r="D2" s="19" t="n"/>
-      <c r="E2" s="19" t="n"/>
-      <c r="F2" s="21" t="n"/>
-      <c r="G2" s="21" t="n"/>
-      <c r="H2" s="21" t="n"/>
+      <c r="C2" s="18" t="n"/>
+      <c r="D2" s="18" t="n"/>
+      <c r="E2" s="20" t="n"/>
+      <c r="F2" s="20" t="n"/>
+      <c r="G2" s="20" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="n">
-        <v>7</v>
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>the clerk / let / me / try on / the scarf</t>
+        </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>the clerk / let / me / try on / the scarf</t>
+          <t>점원은 내가 그 스카프를 착용해 보게 해 주었다.</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>점원은 내가 그 스카프를 착용해 보게 해 주었다.</t>
-        </is>
-      </c>
-      <c r="D3" s="14" t="inlineStr">
-        <is>
           <t>let + 목적어 + 동사원형</t>
         </is>
       </c>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="17" t="n"/>
-      <c r="G3" s="16" t="n"/>
-      <c r="H3" s="17" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="17" t="n"/>
+      <c r="F3" s="16" t="n"/>
+      <c r="G3" s="17" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="n">
-        <v>17</v>
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>I / can / solve / the puzzle / as / easily / as / you</t>
+        </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>I / can / solve / the puzzle / as / easily / as / you</t>
+          <t>나는 너만큼 쉽게 그 퍼즐을 풀 수 있다.</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>나는 너만큼 쉽게 그 퍼즐을 풀 수 있다.</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
           <t>as + 부사 원급 + as</t>
         </is>
       </c>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="17" t="n"/>
-      <c r="G4" s="16" t="n"/>
-      <c r="H4" s="17" t="n"/>
+      <c r="D4" s="14" t="n"/>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="17" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="n">
-        <v>20</v>
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>these sneakers / are / not / as / expensive / as / those boots</t>
+        </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>these sneakers / are / not / as / expensive / as / those boots</t>
+          <t>이 운동화는 저 부츠만큼 비싸지 않다.</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>이 운동화는 저 부츠만큼 비싸지 않다.</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
           <t>not as + 원급 + as</t>
         </is>
       </c>
-      <c r="E5" s="14" t="n"/>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="16" t="n"/>
-      <c r="H5" s="17" t="n"/>
+      <c r="D5" s="14" t="n"/>
+      <c r="E5" s="17" t="n"/>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="17" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="상태" error="사용, 검토, 보관 중에서 고르세요." type="list">
+    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="상태" error="사용, 검토, 보관 중에서 고르세요." type="list">
       <formula1>"사용,검토,보관"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="시간(초)" error="5~60 사이의 숫자를 쓰거나 비워 두세요." type="whole" operator="between">
+    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="시간(초)" error="5~60 사이의 숫자를 쓰거나 비워 두세요." type="whole" operator="between">
       <formula1>5</formula1>
       <formula2>60</formula2>
     </dataValidation>
@@ -3339,483 +3195,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:P21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="9" customWidth="1" style="8" min="1" max="1"/>
-    <col width="40" customWidth="1" style="3" min="2" max="2"/>
-    <col width="14" customWidth="1" style="3" min="3" max="3"/>
-    <col width="14" customWidth="1" style="3" min="4" max="4"/>
-    <col width="14" customWidth="1" style="3" min="5" max="5"/>
-    <col width="14" customWidth="1" style="3" min="6" max="6"/>
-    <col width="9" customWidth="1" style="8" min="7" max="7"/>
-    <col width="28" customWidth="1" style="3" min="8" max="8"/>
-    <col hidden="1" outlineLevel="1" width="8" customWidth="1" style="9" min="9" max="16"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>유형</t>
-        </is>
-      </c>
-      <c r="B1" s="10" t="inlineStr">
-        <is>
-          <t>문제</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>보기1</t>
-        </is>
-      </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>보기2</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
-          <t>보기3</t>
-        </is>
-      </c>
-      <c r="F1" s="11" t="inlineStr">
-        <is>
-          <t>보기4</t>
-        </is>
-      </c>
-      <c r="G1" s="10" t="inlineStr">
-        <is>
-          <t>정답</t>
-        </is>
-      </c>
-      <c r="H1" s="11" t="inlineStr">
-        <is>
-          <t>해설</t>
-        </is>
-      </c>
-      <c r="I1" s="12" t="inlineStr">
-        <is>
-          <t>문항ID</t>
-        </is>
-      </c>
-      <c r="J1" s="12" t="inlineStr">
-        <is>
-          <t>피드백1</t>
-        </is>
-      </c>
-      <c r="K1" s="12" t="inlineStr">
-        <is>
-          <t>피드백2</t>
-        </is>
-      </c>
-      <c r="L1" s="12" t="inlineStr">
-        <is>
-          <t>피드백3</t>
-        </is>
-      </c>
-      <c r="M1" s="12" t="inlineStr">
-        <is>
-          <t>피드백4</t>
-        </is>
-      </c>
-      <c r="N1" s="12" t="inlineStr">
-        <is>
-          <t>시간(초)</t>
-        </is>
-      </c>
-      <c r="O1" s="12" t="inlineStr">
-        <is>
-          <t>세트</t>
-        </is>
-      </c>
-      <c r="P1" s="12" t="inlineStr">
-        <is>
-          <t>상태</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="15" t="n"/>
-      <c r="B2" s="14" t="n"/>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="14" t="n"/>
-      <c r="G2" s="15" t="n"/>
-      <c r="H2" s="14" t="n"/>
-      <c r="I2" s="16" t="n"/>
-      <c r="J2" s="23" t="n"/>
-      <c r="K2" s="23" t="n"/>
-      <c r="L2" s="23" t="n"/>
-      <c r="M2" s="23" t="n"/>
-      <c r="N2" s="17" t="n"/>
-      <c r="O2" s="16" t="n"/>
-      <c r="P2" s="17" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="15" t="n"/>
-      <c r="B3" s="14" t="n"/>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="14" t="n"/>
-      <c r="G3" s="15" t="n"/>
-      <c r="H3" s="14" t="n"/>
-      <c r="I3" s="16" t="n"/>
-      <c r="J3" s="23" t="n"/>
-      <c r="K3" s="23" t="n"/>
-      <c r="L3" s="23" t="n"/>
-      <c r="M3" s="23" t="n"/>
-      <c r="N3" s="17" t="n"/>
-      <c r="O3" s="16" t="n"/>
-      <c r="P3" s="17" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="15" t="n"/>
-      <c r="B4" s="14" t="n"/>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="14" t="n"/>
-      <c r="G4" s="15" t="n"/>
-      <c r="H4" s="14" t="n"/>
-      <c r="I4" s="16" t="n"/>
-      <c r="J4" s="23" t="n"/>
-      <c r="K4" s="23" t="n"/>
-      <c r="L4" s="23" t="n"/>
-      <c r="M4" s="23" t="n"/>
-      <c r="N4" s="17" t="n"/>
-      <c r="O4" s="16" t="n"/>
-      <c r="P4" s="17" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="15" t="n"/>
-      <c r="B5" s="14" t="n"/>
-      <c r="C5" s="14" t="n"/>
-      <c r="D5" s="14" t="n"/>
-      <c r="E5" s="14" t="n"/>
-      <c r="F5" s="14" t="n"/>
-      <c r="G5" s="15" t="n"/>
-      <c r="H5" s="14" t="n"/>
-      <c r="I5" s="16" t="n"/>
-      <c r="J5" s="23" t="n"/>
-      <c r="K5" s="23" t="n"/>
-      <c r="L5" s="23" t="n"/>
-      <c r="M5" s="23" t="n"/>
-      <c r="N5" s="17" t="n"/>
-      <c r="O5" s="16" t="n"/>
-      <c r="P5" s="17" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="n"/>
-      <c r="B6" s="14" t="n"/>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="14" t="n"/>
-      <c r="E6" s="14" t="n"/>
-      <c r="F6" s="14" t="n"/>
-      <c r="G6" s="15" t="n"/>
-      <c r="H6" s="14" t="n"/>
-      <c r="I6" s="16" t="n"/>
-      <c r="J6" s="23" t="n"/>
-      <c r="K6" s="23" t="n"/>
-      <c r="L6" s="23" t="n"/>
-      <c r="M6" s="23" t="n"/>
-      <c r="N6" s="17" t="n"/>
-      <c r="O6" s="16" t="n"/>
-      <c r="P6" s="17" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="n"/>
-      <c r="B7" s="14" t="n"/>
-      <c r="C7" s="14" t="n"/>
-      <c r="D7" s="14" t="n"/>
-      <c r="E7" s="14" t="n"/>
-      <c r="F7" s="14" t="n"/>
-      <c r="G7" s="15" t="n"/>
-      <c r="H7" s="14" t="n"/>
-      <c r="I7" s="16" t="n"/>
-      <c r="J7" s="23" t="n"/>
-      <c r="K7" s="23" t="n"/>
-      <c r="L7" s="23" t="n"/>
-      <c r="M7" s="23" t="n"/>
-      <c r="N7" s="17" t="n"/>
-      <c r="O7" s="16" t="n"/>
-      <c r="P7" s="17" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="n"/>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="n"/>
-      <c r="E8" s="14" t="n"/>
-      <c r="F8" s="14" t="n"/>
-      <c r="G8" s="15" t="n"/>
-      <c r="H8" s="14" t="n"/>
-      <c r="I8" s="16" t="n"/>
-      <c r="J8" s="23" t="n"/>
-      <c r="K8" s="23" t="n"/>
-      <c r="L8" s="23" t="n"/>
-      <c r="M8" s="23" t="n"/>
-      <c r="N8" s="17" t="n"/>
-      <c r="O8" s="16" t="n"/>
-      <c r="P8" s="17" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="n"/>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="14" t="n"/>
-      <c r="E9" s="14" t="n"/>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="15" t="n"/>
-      <c r="H9" s="14" t="n"/>
-      <c r="I9" s="16" t="n"/>
-      <c r="J9" s="23" t="n"/>
-      <c r="K9" s="23" t="n"/>
-      <c r="L9" s="23" t="n"/>
-      <c r="M9" s="23" t="n"/>
-      <c r="N9" s="17" t="n"/>
-      <c r="O9" s="16" t="n"/>
-      <c r="P9" s="17" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="n"/>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="14" t="n"/>
-      <c r="E10" s="14" t="n"/>
-      <c r="F10" s="14" t="n"/>
-      <c r="G10" s="15" t="n"/>
-      <c r="H10" s="14" t="n"/>
-      <c r="I10" s="16" t="n"/>
-      <c r="J10" s="23" t="n"/>
-      <c r="K10" s="23" t="n"/>
-      <c r="L10" s="23" t="n"/>
-      <c r="M10" s="23" t="n"/>
-      <c r="N10" s="17" t="n"/>
-      <c r="O10" s="16" t="n"/>
-      <c r="P10" s="17" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="15" t="n"/>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="14" t="n"/>
-      <c r="E11" s="14" t="n"/>
-      <c r="F11" s="14" t="n"/>
-      <c r="G11" s="15" t="n"/>
-      <c r="H11" s="14" t="n"/>
-      <c r="I11" s="16" t="n"/>
-      <c r="J11" s="23" t="n"/>
-      <c r="K11" s="23" t="n"/>
-      <c r="L11" s="23" t="n"/>
-      <c r="M11" s="23" t="n"/>
-      <c r="N11" s="17" t="n"/>
-      <c r="O11" s="16" t="n"/>
-      <c r="P11" s="17" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="15" t="n"/>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="14" t="n"/>
-      <c r="E12" s="14" t="n"/>
-      <c r="F12" s="14" t="n"/>
-      <c r="G12" s="15" t="n"/>
-      <c r="H12" s="14" t="n"/>
-      <c r="I12" s="16" t="n"/>
-      <c r="J12" s="23" t="n"/>
-      <c r="K12" s="23" t="n"/>
-      <c r="L12" s="23" t="n"/>
-      <c r="M12" s="23" t="n"/>
-      <c r="N12" s="17" t="n"/>
-      <c r="O12" s="16" t="n"/>
-      <c r="P12" s="17" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="n"/>
-      <c r="B13" s="14" t="n"/>
-      <c r="C13" s="14" t="n"/>
-      <c r="D13" s="14" t="n"/>
-      <c r="E13" s="14" t="n"/>
-      <c r="F13" s="14" t="n"/>
-      <c r="G13" s="15" t="n"/>
-      <c r="H13" s="14" t="n"/>
-      <c r="I13" s="16" t="n"/>
-      <c r="J13" s="23" t="n"/>
-      <c r="K13" s="23" t="n"/>
-      <c r="L13" s="23" t="n"/>
-      <c r="M13" s="23" t="n"/>
-      <c r="N13" s="17" t="n"/>
-      <c r="O13" s="16" t="n"/>
-      <c r="P13" s="17" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="n"/>
-      <c r="B14" s="14" t="n"/>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="14" t="n"/>
-      <c r="E14" s="14" t="n"/>
-      <c r="F14" s="14" t="n"/>
-      <c r="G14" s="15" t="n"/>
-      <c r="H14" s="14" t="n"/>
-      <c r="I14" s="16" t="n"/>
-      <c r="J14" s="23" t="n"/>
-      <c r="K14" s="23" t="n"/>
-      <c r="L14" s="23" t="n"/>
-      <c r="M14" s="23" t="n"/>
-      <c r="N14" s="17" t="n"/>
-      <c r="O14" s="16" t="n"/>
-      <c r="P14" s="17" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="n"/>
-      <c r="B15" s="14" t="n"/>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="14" t="n"/>
-      <c r="E15" s="14" t="n"/>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="15" t="n"/>
-      <c r="H15" s="14" t="n"/>
-      <c r="I15" s="16" t="n"/>
-      <c r="J15" s="23" t="n"/>
-      <c r="K15" s="23" t="n"/>
-      <c r="L15" s="23" t="n"/>
-      <c r="M15" s="23" t="n"/>
-      <c r="N15" s="17" t="n"/>
-      <c r="O15" s="16" t="n"/>
-      <c r="P15" s="17" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="n"/>
-      <c r="B16" s="14" t="n"/>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="14" t="n"/>
-      <c r="E16" s="14" t="n"/>
-      <c r="F16" s="14" t="n"/>
-      <c r="G16" s="15" t="n"/>
-      <c r="H16" s="14" t="n"/>
-      <c r="I16" s="16" t="n"/>
-      <c r="J16" s="23" t="n"/>
-      <c r="K16" s="23" t="n"/>
-      <c r="L16" s="23" t="n"/>
-      <c r="M16" s="23" t="n"/>
-      <c r="N16" s="17" t="n"/>
-      <c r="O16" s="16" t="n"/>
-      <c r="P16" s="17" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="n"/>
-      <c r="B17" s="14" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="14" t="n"/>
-      <c r="E17" s="14" t="n"/>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="15" t="n"/>
-      <c r="H17" s="14" t="n"/>
-      <c r="I17" s="16" t="n"/>
-      <c r="J17" s="23" t="n"/>
-      <c r="K17" s="23" t="n"/>
-      <c r="L17" s="23" t="n"/>
-      <c r="M17" s="23" t="n"/>
-      <c r="N17" s="17" t="n"/>
-      <c r="O17" s="16" t="n"/>
-      <c r="P17" s="17" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="n"/>
-      <c r="B18" s="14" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="14" t="n"/>
-      <c r="E18" s="14" t="n"/>
-      <c r="F18" s="14" t="n"/>
-      <c r="G18" s="15" t="n"/>
-      <c r="H18" s="14" t="n"/>
-      <c r="I18" s="16" t="n"/>
-      <c r="J18" s="23" t="n"/>
-      <c r="K18" s="23" t="n"/>
-      <c r="L18" s="23" t="n"/>
-      <c r="M18" s="23" t="n"/>
-      <c r="N18" s="17" t="n"/>
-      <c r="O18" s="16" t="n"/>
-      <c r="P18" s="17" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="15" t="n"/>
-      <c r="B19" s="14" t="n"/>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="14" t="n"/>
-      <c r="E19" s="14" t="n"/>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="15" t="n"/>
-      <c r="H19" s="14" t="n"/>
-      <c r="I19" s="16" t="n"/>
-      <c r="J19" s="23" t="n"/>
-      <c r="K19" s="23" t="n"/>
-      <c r="L19" s="23" t="n"/>
-      <c r="M19" s="23" t="n"/>
-      <c r="N19" s="17" t="n"/>
-      <c r="O19" s="16" t="n"/>
-      <c r="P19" s="17" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="15" t="n"/>
-      <c r="B20" s="14" t="n"/>
-      <c r="C20" s="14" t="n"/>
-      <c r="D20" s="14" t="n"/>
-      <c r="E20" s="14" t="n"/>
-      <c r="F20" s="14" t="n"/>
-      <c r="G20" s="15" t="n"/>
-      <c r="H20" s="14" t="n"/>
-      <c r="I20" s="16" t="n"/>
-      <c r="J20" s="23" t="n"/>
-      <c r="K20" s="23" t="n"/>
-      <c r="L20" s="23" t="n"/>
-      <c r="M20" s="23" t="n"/>
-      <c r="N20" s="17" t="n"/>
-      <c r="O20" s="16" t="n"/>
-      <c r="P20" s="17" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="n"/>
-      <c r="B21" s="14" t="n"/>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="14" t="n"/>
-      <c r="E21" s="14" t="n"/>
-      <c r="F21" s="14" t="n"/>
-      <c r="G21" s="15" t="n"/>
-      <c r="H21" s="14" t="n"/>
-      <c r="I21" s="16" t="n"/>
-      <c r="J21" s="23" t="n"/>
-      <c r="K21" s="23" t="n"/>
-      <c r="L21" s="23" t="n"/>
-      <c r="M21" s="23" t="n"/>
-      <c r="N21" s="17" t="n"/>
-      <c r="O21" s="16" t="n"/>
-      <c r="P21" s="17" t="n"/>
-    </row>
-  </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="P2:P500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="상태" error="사용, 검토, 보관 중에서 고르세요." type="list">
-      <formula1>"사용,검토,보관"</formula1>
-    </dataValidation>
-    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="시간(초)" error="5~60 사이의 숫자를 쓰거나 비워 두세요." type="whole" operator="between">
-      <formula1>5</formula1>
-      <formula2>60</formula2>
-    </dataValidation>
-    <dataValidation sqref="A2:A500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="유형" error="객관식, OX, 단답형 중에서 고르세요." type="list">
-      <formula1>"객관식,OX,단답형"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>